<commit_message>
chore: update latest generated excel report files
- Update General Ledger
- Update Journal
- Update Worksheet
- Update other outputs
</commit_message>
<xml_diff>
--- a/output-app/BUKU BESAR 2026.xlsx
+++ b/output-app/BUKU BESAR 2026.xlsx
@@ -5,7 +5,13 @@
   <sheets>
     <sheet name="11.01.00" sheetId="1" r:id="rId1"/>
     <sheet name="13.01.00" sheetId="2" r:id="rId2"/>
-    <sheet name="81.02.50" sheetId="3" r:id="rId3"/>
+    <sheet name="15.01.00" sheetId="3" r:id="rId3"/>
+    <sheet name="15.03.00" sheetId="4" r:id="rId4"/>
+    <sheet name="50.01.00" sheetId="5" r:id="rId5"/>
+    <sheet name="50.01.01" sheetId="6" r:id="rId6"/>
+    <sheet name="71.01.00" sheetId="7" r:id="rId7"/>
+    <sheet name="81.02.50" sheetId="8" r:id="rId8"/>
+    <sheet name="97.06.20" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -407,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
@@ -559,22 +565,22 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>18 Mei 2026</v>
+        <v>02 Jan 2001</v>
       </c>
       <c r="B8" t="str">
-        <v>Penerimaan Rek Air (KOPERASI)</v>
+        <v>Bayar: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
       </c>
       <c r="C8" t="str">
         <v>JPK</v>
       </c>
-      <c r="D8">
-        <v>79000</v>
-      </c>
-      <c r="E8" t="str">
-        <v/>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8">
+        <v>200000</v>
       </c>
       <c r="F8">
-        <v>79000</v>
+        <v>-200000</v>
       </c>
     </row>
     <row r="9">
@@ -582,19 +588,19 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B9" t="str">
-        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+        <v>Penerimaan Rek Air (KOPERASI)</v>
       </c>
       <c r="C9" t="str">
         <v>JPK</v>
       </c>
       <c r="D9">
-        <v>361700</v>
+        <v>79000</v>
       </c>
       <c r="E9" t="str">
         <v/>
       </c>
       <c r="F9">
-        <v>440700</v>
+        <v>-121000</v>
       </c>
     </row>
     <row r="10">
@@ -602,19 +608,19 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B10" t="str">
-        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
       </c>
       <c r="C10" t="str">
         <v>JPK</v>
       </c>
       <c r="D10">
-        <v>302900</v>
+        <v>361700</v>
       </c>
       <c r="E10" t="str">
         <v/>
       </c>
       <c r="F10">
-        <v>743600</v>
+        <v>240700</v>
       </c>
     </row>
     <row r="11">
@@ -622,19 +628,19 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B11" t="str">
-        <v>Penerimaan Rek Air (KOPERASI)</v>
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
       </c>
       <c r="C11" t="str">
         <v>JPK</v>
       </c>
       <c r="D11">
-        <v>79000</v>
+        <v>302900</v>
       </c>
       <c r="E11" t="str">
         <v/>
       </c>
       <c r="F11">
-        <v>822600</v>
+        <v>543600</v>
       </c>
     </row>
     <row r="12">
@@ -642,19 +648,19 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B12" t="str">
-        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+        <v>Penerimaan Rek Air (KOPERASI)</v>
       </c>
       <c r="C12" t="str">
         <v>JPK</v>
       </c>
       <c r="D12">
-        <v>361700</v>
+        <v>79000</v>
       </c>
       <c r="E12" t="str">
         <v/>
       </c>
       <c r="F12">
-        <v>1184300</v>
+        <v>622600</v>
       </c>
     </row>
     <row r="13">
@@ -662,19 +668,19 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B13" t="str">
-        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
       </c>
       <c r="C13" t="str">
         <v>JPK</v>
       </c>
       <c r="D13">
-        <v>302900</v>
+        <v>361700</v>
       </c>
       <c r="E13" t="str">
         <v/>
       </c>
       <c r="F13">
-        <v>1487200</v>
+        <v>984300</v>
       </c>
     </row>
     <row r="14">
@@ -682,19 +688,19 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B14" t="str">
-        <v>Penerimaan Rek Air (KOPERASI)</v>
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
       </c>
       <c r="C14" t="str">
         <v>JPK</v>
       </c>
       <c r="D14">
-        <v>79000</v>
+        <v>302900</v>
       </c>
       <c r="E14" t="str">
         <v/>
       </c>
       <c r="F14">
-        <v>1566200</v>
+        <v>1287200</v>
       </c>
     </row>
     <row r="15">
@@ -702,19 +708,19 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B15" t="str">
-        <v>Penerimaan Rek Air (LOKET CABANG)</v>
+        <v>Penerimaan Rek Air (KOPERASI)</v>
       </c>
       <c r="C15" t="str">
         <v>JPK</v>
       </c>
       <c r="D15">
-        <v>361700</v>
+        <v>79000</v>
       </c>
       <c r="E15" t="str">
         <v/>
       </c>
       <c r="F15">
-        <v>1927900</v>
+        <v>1366200</v>
       </c>
     </row>
     <row r="16">
@@ -722,64 +728,104 @@
         <v>18 Mei 2026</v>
       </c>
       <c r="B16" t="str">
-        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
+        <v>Penerimaan Rek Air (LOKET CABANG)</v>
       </c>
       <c r="C16" t="str">
         <v>JPK</v>
       </c>
       <c r="D16">
-        <v>302900</v>
+        <v>361700</v>
       </c>
       <c r="E16" t="str">
         <v/>
       </c>
       <c r="F16">
-        <v>2230800</v>
+        <v>1727900</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>18 Mei 2026</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>Penerimaan Rek Air (LOKET KANTOR)</v>
       </c>
       <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v/>
+        <v>JPK</v>
+      </c>
+      <c r="D17">
+        <v>302900</v>
       </c>
       <c r="E17" t="str">
         <v/>
       </c>
-      <c r="F17" t="str">
-        <v/>
+      <c r="F17">
+        <v>2030800</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Bayar: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="C18" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18">
+        <v>125000</v>
+      </c>
+      <c r="F18">
+        <v>1905800</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>JUMLAH MUTASI</v>
       </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18">
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20">
         <v>2230800</v>
       </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-      <c r="F18">
-        <v>2230800</v>
+      <c r="E20">
+        <v>325000</v>
+      </c>
+      <c r="F20">
+        <v>1905800</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1165,6 +1211,1181 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F11"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PERUSAHAAN DAERAH AIR MINUM</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>KABUPATEN SERUYAN</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BUKU BESAR</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Nama Perk : Persediaan Bahan Kimia</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Kode Perkiraan : 15.01.00</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tgl</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Uraian</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ref.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mutasi</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Saldo Akhir</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Debet</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Kredit</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>01 Jan 2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Persediaan Bahan Kimia &amp; BBM</v>
+      </c>
+      <c r="C8" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D8">
+        <v>644</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="C9" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D9">
+        <v>125000</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9">
+        <v>125644</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>JUMLAH MUTASI</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11">
+        <v>125644</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>125644</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F10"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PERUSAHAAN DAERAH AIR MINUM</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>KABUPATEN SERUYAN</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BUKU BESAR</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Nama Perk : Persediaan Bahan Instalasi</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Kode Perkiraan : 15.03.00</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tgl</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Uraian</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ref.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mutasi</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Saldo Akhir</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Debet</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Kredit</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>01 Jan 2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Persediaan Bahan Instalasi (Asesoris &amp; Water Meter)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D8">
+        <v>21696230000.277004</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8">
+        <v>21696230000.28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>JUMLAH MUTASI</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10">
+        <v>21696230000.277004</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>21696230000.28</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F12"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PERUSAHAAN DAERAH AIR MINUM</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>KABUPATEN SERUYAN</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BUKU BESAR</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Nama Perk : Utang Usaha</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Kode Perkiraan : 50.01.00</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tgl</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Uraian</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ref.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mutasi</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Saldo Akhir</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Debet</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Kredit</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>02 Jan 2001</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="C8" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8">
+        <v>200000</v>
+      </c>
+      <c r="F8">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>02 Jan 2001</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bayar: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="C9" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D9">
+        <v>200000</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Bayar: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="C10" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D10">
+        <v>125000</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10">
+        <v>-125000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>JUMLAH MUTASI</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12">
+        <v>325000</v>
+      </c>
+      <c r="E12">
+        <v>200000</v>
+      </c>
+      <c r="F12">
+        <v>-125000</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F10"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PERUSAHAAN DAERAH AIR MINUM</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>KABUPATEN SERUYAN</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BUKU BESAR</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Nama Perk : Utang Usaha - Bahan Kimia</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Kode Perkiraan : 50.01.01</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tgl</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Uraian</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ref.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mutasi</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Saldo Akhir</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Debet</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Kredit</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>21 Jan 2001</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Voucher: Pembayaran Belanja Bahan Habis Pakai Tawas dll</v>
+      </c>
+      <c r="C8" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8">
+        <v>125000</v>
+      </c>
+      <c r="F8">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>JUMLAH MUTASI</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>125000</v>
+      </c>
+      <c r="F10">
+        <v>125000</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F11"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PERUSAHAAN DAERAH AIR MINUM</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>KABUPATEN SERUYAN</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BUKU BESAR</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Nama Perk : Kekayaan Pemda Yang Dipisahkan</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Kode Perkiraan : 71.01.00</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tgl</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Uraian</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ref.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mutasi</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Saldo Akhir</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Debet</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Kredit</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>01 Jan 2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Persediaan Bahan Instalasi (Asesoris &amp; Water Meter)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8">
+        <v>21696230000.277004</v>
+      </c>
+      <c r="F8">
+        <v>21696230000.28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>01 Jan 2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Persediaan Bahan Kimia &amp; BBM</v>
+      </c>
+      <c r="C9" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9">
+        <v>644</v>
+      </c>
+      <c r="F9">
+        <v>21696230644.28</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>JUMLAH MUTASI</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>21696230644.277004</v>
+      </c>
+      <c r="F11">
+        <v>21696230644.28</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F18"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
@@ -1540,4 +2761,223 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F10"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PERUSAHAAN DAERAH AIR MINUM</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>KABUPATEN SERUYAN</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BUKU BESAR</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Nama Perk : Pemeliharaan Kendaraan</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Kode Perkiraan : 97.06.20</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tgl</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Uraian</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ref.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mutasi</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Saldo Akhir</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Debet</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Kredit</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>02 Jan 2001</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Voucher: Pembayaran Biaya Perpanjangan STNK Mobil Pick Up KH 1234 PU</v>
+      </c>
+      <c r="C8" t="str">
+        <v>JPK</v>
+      </c>
+      <c r="D8">
+        <v>200000</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>JUMLAH MUTASI</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10">
+        <v>200000</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>200000</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>